<commit_message>
04/03/2026 - Observaciones completadas
</commit_message>
<xml_diff>
--- a/plantillas/Incidentes.xlsx
+++ b/plantillas/Incidentes.xlsx
@@ -1,9 +1,9 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29725"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FC8529F3-DFD2-4EA7-856C-3AE94720DFD9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{20C5A16C-7B90-44E5-8C62-A3C7B8222D6C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -313,7 +313,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="38">
+  <cellXfs count="37">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -349,9 +349,6 @@
     <xf numFmtId="0" fontId="13" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -365,10 +362,6 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
@@ -379,12 +372,11 @@
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="12" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -392,6 +384,15 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="2" borderId="9" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1162,27 +1163,27 @@
     <col min="16146" max="16146" width="27.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:34" s="26" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B1" s="29"/>
-      <c r="C1" s="29"/>
-      <c r="D1" s="29"/>
-      <c r="E1" s="29"/>
-      <c r="F1" s="29"/>
-      <c r="G1" s="29"/>
-      <c r="H1" s="29"/>
-      <c r="I1" s="29"/>
-      <c r="J1" s="29"/>
-      <c r="K1" s="29"/>
-      <c r="L1" s="29"/>
-      <c r="M1" s="29"/>
-      <c r="N1" s="29"/>
-      <c r="O1" s="29"/>
-      <c r="P1" s="29"/>
-      <c r="Q1" s="29"/>
-      <c r="R1" s="29"/>
+    <row r="1" spans="1:34" x14ac:dyDescent="0.25">
+      <c r="B1" s="26"/>
+      <c r="C1" s="26"/>
+      <c r="D1" s="26"/>
+      <c r="E1" s="26"/>
+      <c r="F1" s="26"/>
+      <c r="G1" s="26"/>
+      <c r="H1" s="26"/>
+      <c r="I1" s="26"/>
+      <c r="J1" s="26"/>
+      <c r="K1" s="26"/>
+      <c r="L1" s="26"/>
+      <c r="M1" s="26"/>
+      <c r="N1" s="26"/>
+      <c r="O1" s="26"/>
+      <c r="P1" s="26"/>
+      <c r="Q1" s="26"/>
+      <c r="R1" s="26"/>
     </row>
     <row r="2" spans="1:34" ht="20.25" x14ac:dyDescent="0.25">
-      <c r="A2" s="23"/>
+      <c r="A2" s="22"/>
       <c r="B2" s="5"/>
       <c r="C2" s="15"/>
       <c r="D2" s="15"/>
@@ -1201,9 +1202,9 @@
       <c r="Q2" s="15"/>
       <c r="R2" s="15"/>
     </row>
-    <row r="3" spans="1:34" ht="20.25" x14ac:dyDescent="0.25">
-      <c r="A3" s="21"/>
-      <c r="B3" s="25"/>
+    <row r="3" spans="1:34" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="35"/>
+      <c r="B3" s="36"/>
       <c r="C3" s="15"/>
       <c r="D3" s="15"/>
       <c r="E3" s="15"/>
@@ -1221,48 +1222,48 @@
       <c r="Q3" s="15"/>
       <c r="R3" s="15"/>
     </row>
-    <row r="4" spans="1:34" s="26" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B4" s="30"/>
-      <c r="C4" s="30"/>
-      <c r="D4" s="30"/>
-      <c r="E4" s="30"/>
-      <c r="F4" s="30"/>
-      <c r="G4" s="30"/>
-      <c r="H4" s="30"/>
-      <c r="I4" s="30"/>
-      <c r="J4" s="30"/>
-      <c r="K4" s="30"/>
-      <c r="L4" s="30"/>
-      <c r="M4" s="30"/>
-      <c r="N4" s="30"/>
-      <c r="O4" s="30"/>
-      <c r="P4" s="30"/>
-      <c r="Q4" s="30"/>
-      <c r="R4" s="30"/>
+    <row r="4" spans="1:34" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B4" s="27"/>
+      <c r="C4" s="27"/>
+      <c r="D4" s="27"/>
+      <c r="E4" s="27"/>
+      <c r="F4" s="27"/>
+      <c r="G4" s="27"/>
+      <c r="H4" s="27"/>
+      <c r="I4" s="27"/>
+      <c r="J4" s="27"/>
+      <c r="K4" s="27"/>
+      <c r="L4" s="27"/>
+      <c r="M4" s="27"/>
+      <c r="N4" s="27"/>
+      <c r="O4" s="27"/>
+      <c r="P4" s="27"/>
+      <c r="Q4" s="27"/>
+      <c r="R4" s="27"/>
     </row>
     <row r="5" spans="1:34" s="4" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="21"/>
-      <c r="B5" s="21"/>
-      <c r="C5" s="20"/>
-      <c r="D5" s="20"/>
-      <c r="E5" s="20"/>
-      <c r="F5" s="20"/>
-      <c r="G5" s="20"/>
-      <c r="H5" s="20"/>
-      <c r="I5" s="20"/>
-      <c r="J5" s="20"/>
-      <c r="K5" s="20"/>
-      <c r="L5" s="20"/>
-      <c r="M5" s="20"/>
-      <c r="N5" s="20"/>
-      <c r="O5" s="20"/>
+      <c r="A5" s="20"/>
+      <c r="B5" s="20"/>
+      <c r="C5" s="19"/>
+      <c r="D5" s="19"/>
+      <c r="E5" s="19"/>
+      <c r="F5" s="19"/>
+      <c r="G5" s="19"/>
+      <c r="H5" s="19"/>
+      <c r="I5" s="19"/>
+      <c r="J5" s="19"/>
+      <c r="K5" s="19"/>
+      <c r="L5" s="19"/>
+      <c r="M5" s="19"/>
+      <c r="N5" s="19"/>
+      <c r="O5" s="19"/>
       <c r="P5" s="16"/>
       <c r="Q5" s="16"/>
       <c r="R5" s="16"/>
     </row>
     <row r="6" spans="1:34" ht="18" x14ac:dyDescent="0.25">
-      <c r="A6" s="21"/>
-      <c r="B6" s="21"/>
+      <c r="A6" s="20"/>
+      <c r="B6" s="20"/>
       <c r="C6" s="2"/>
       <c r="D6" s="2"/>
       <c r="E6" s="2"/>
@@ -1275,26 +1276,26 @@
       <c r="L6" s="2"/>
       <c r="M6" s="2"/>
       <c r="N6" s="2"/>
-      <c r="O6" s="24"/>
+      <c r="O6" s="23"/>
       <c r="P6" s="2"/>
     </row>
-    <row r="7" spans="1:34" s="26" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="C7" s="33"/>
-      <c r="D7" s="33"/>
-      <c r="E7" s="33"/>
-      <c r="F7" s="33"/>
-      <c r="G7" s="33"/>
-      <c r="H7" s="33"/>
-      <c r="I7" s="33"/>
-      <c r="J7" s="33"/>
-      <c r="K7" s="33"/>
-      <c r="L7" s="33"/>
-      <c r="M7" s="33"/>
-      <c r="N7" s="33"/>
-      <c r="O7" s="33"/>
-      <c r="P7" s="34"/>
-      <c r="Q7" s="34"/>
-      <c r="R7" s="34"/>
+    <row r="7" spans="1:34" x14ac:dyDescent="0.25">
+      <c r="C7" s="30"/>
+      <c r="D7" s="30"/>
+      <c r="E7" s="30"/>
+      <c r="F7" s="30"/>
+      <c r="G7" s="30"/>
+      <c r="H7" s="30"/>
+      <c r="I7" s="30"/>
+      <c r="J7" s="30"/>
+      <c r="K7" s="30"/>
+      <c r="L7" s="30"/>
+      <c r="M7" s="30"/>
+      <c r="N7" s="30"/>
+      <c r="O7" s="30"/>
+      <c r="P7" s="28"/>
+      <c r="Q7" s="28"/>
+      <c r="R7" s="28"/>
       <c r="S7" s="3"/>
       <c r="T7" s="3"/>
       <c r="U7" s="3"/>
@@ -1313,7 +1314,8 @@
       <c r="AH7" s="3"/>
     </row>
     <row r="8" spans="1:34" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B8" s="19"/>
+      <c r="A8" s="34"/>
+      <c r="B8" s="34"/>
       <c r="C8" s="14"/>
       <c r="D8" s="3"/>
       <c r="E8" s="3"/>
@@ -1324,72 +1326,74 @@
       <c r="J8" s="3"/>
       <c r="K8" s="3"/>
       <c r="L8" s="1"/>
-      <c r="M8" s="32"/>
-      <c r="N8" s="7" t="s">
+      <c r="M8" s="29"/>
+      <c r="N8" s="7"/>
+      <c r="O8" s="7" t="s">
         <v>6</v>
       </c>
       <c r="R8" s="6"/>
     </row>
     <row r="9" spans="1:34" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="G9" s="31"/>
-      <c r="H9" s="31"/>
-      <c r="I9" s="31"/>
-      <c r="J9" s="31"/>
-      <c r="K9" s="31"/>
-      <c r="N9" s="17" t="s">
+      <c r="G9" s="28"/>
+      <c r="H9" s="28"/>
+      <c r="I9" s="28"/>
+      <c r="J9" s="28"/>
+      <c r="K9" s="28"/>
+      <c r="N9" s="17"/>
+      <c r="O9" s="17" t="s">
         <v>7</v>
       </c>
       <c r="P9" s="6"/>
     </row>
-    <row r="10" spans="1:34" s="26" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="G10" s="31"/>
-      <c r="H10" s="31"/>
-      <c r="I10" s="31"/>
-      <c r="J10" s="31"/>
-      <c r="K10" s="31"/>
-      <c r="L10" s="27"/>
-      <c r="P10" s="28"/>
-    </row>
-    <row r="11" spans="1:34" s="26" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="35" t="s">
+    <row r="10" spans="1:34" x14ac:dyDescent="0.25">
+      <c r="G10" s="28"/>
+      <c r="H10" s="28"/>
+      <c r="I10" s="28"/>
+      <c r="J10" s="28"/>
+      <c r="K10" s="28"/>
+      <c r="L10" s="24"/>
+      <c r="P10" s="25"/>
+    </row>
+    <row r="11" spans="1:34" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="31" t="s">
         <v>13</v>
       </c>
-      <c r="B11" s="37" t="s">
+      <c r="B11" s="33" t="s">
         <v>3</v>
       </c>
-      <c r="C11" s="37" t="s">
+      <c r="C11" s="33" t="s">
         <v>15</v>
       </c>
-      <c r="D11" s="37" t="s">
+      <c r="D11" s="33" t="s">
         <v>5</v>
       </c>
-      <c r="E11" s="37" t="s">
+      <c r="E11" s="33" t="s">
         <v>14</v>
       </c>
-      <c r="F11" s="37" t="s">
+      <c r="F11" s="33" t="s">
         <v>16</v>
       </c>
-      <c r="G11" s="22"/>
-      <c r="H11" s="22"/>
-      <c r="I11" s="22"/>
-      <c r="J11" s="22"/>
-      <c r="K11" s="22"/>
-      <c r="L11" s="37" t="s">
+      <c r="G11" s="21"/>
+      <c r="H11" s="21"/>
+      <c r="I11" s="21"/>
+      <c r="J11" s="21"/>
+      <c r="K11" s="21"/>
+      <c r="L11" s="33" t="s">
         <v>0</v>
       </c>
-      <c r="M11" s="37" t="s">
+      <c r="M11" s="33" t="s">
         <v>2</v>
       </c>
-      <c r="N11" s="37" t="s">
+      <c r="N11" s="33" t="s">
         <v>1</v>
       </c>
-      <c r="O11" s="37" t="s">
+      <c r="O11" s="33" t="s">
         <v>4</v>
       </c>
-      <c r="P11" s="28"/>
+      <c r="P11" s="25"/>
     </row>
     <row r="12" spans="1:34" ht="75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="36"/>
+      <c r="A12" s="32"/>
       <c r="B12" s="18"/>
       <c r="C12" s="18"/>
       <c r="D12" s="18"/>

</xml_diff>

<commit_message>
18/03/2026 - Ultimas observaciones
</commit_message>
<xml_diff>
--- a/plantillas/Incidentes.xlsx
+++ b/plantillas/Incidentes.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29725"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{20C5A16C-7B90-44E5-8C62-A3C7B8222D6C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{46AC8FD2-36F7-425D-8A6C-282FA2AA78B7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -203,7 +203,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="10">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -221,68 +221,6 @@
       <top/>
       <bottom style="thin">
         <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color theme="0" tint="-0.249977111117893"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color theme="0" tint="-0.249977111117893"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color theme="0" tint="-0.249977111117893"/>
-      </right>
-      <top style="thin">
-        <color theme="0" tint="-0.249977111117893"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color theme="0" tint="-0.249977111117893"/>
-      </left>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color theme="0" tint="-0.249977111117893"/>
-      </right>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color theme="0" tint="-0.249977111117893"/>
-      </left>
-      <right/>
-      <top/>
-      <bottom style="thin">
-        <color theme="0" tint="-0.249977111117893"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color theme="0" tint="-0.249977111117893"/>
-      </right>
-      <top/>
-      <bottom style="thin">
-        <color theme="0" tint="-0.249977111117893"/>
       </bottom>
       <diagonal/>
     </border>
@@ -313,7 +251,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="37">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -328,12 +266,6 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -355,7 +287,7 @@
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -377,13 +309,13 @@
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="2" borderId="9" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -395,6 +327,7 @@
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1164,106 +1097,106 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:34" x14ac:dyDescent="0.25">
-      <c r="B1" s="26"/>
-      <c r="C1" s="26"/>
-      <c r="D1" s="26"/>
-      <c r="E1" s="26"/>
-      <c r="F1" s="26"/>
-      <c r="G1" s="26"/>
-      <c r="H1" s="26"/>
-      <c r="I1" s="26"/>
-      <c r="J1" s="26"/>
-      <c r="K1" s="26"/>
-      <c r="L1" s="26"/>
-      <c r="M1" s="26"/>
-      <c r="N1" s="26"/>
-      <c r="O1" s="26"/>
-      <c r="P1" s="26"/>
-      <c r="Q1" s="26"/>
-      <c r="R1" s="26"/>
+      <c r="B1" s="20"/>
+      <c r="C1" s="20"/>
+      <c r="D1" s="20"/>
+      <c r="E1" s="20"/>
+      <c r="F1" s="20"/>
+      <c r="G1" s="20"/>
+      <c r="H1" s="20"/>
+      <c r="I1" s="20"/>
+      <c r="J1" s="20"/>
+      <c r="K1" s="20"/>
+      <c r="L1" s="20"/>
+      <c r="M1" s="20"/>
+      <c r="N1" s="20"/>
+      <c r="O1" s="20"/>
+      <c r="P1" s="20"/>
+      <c r="Q1" s="20"/>
+      <c r="R1" s="20"/>
     </row>
     <row r="2" spans="1:34" ht="20.25" x14ac:dyDescent="0.25">
-      <c r="A2" s="22"/>
+      <c r="A2" s="16"/>
       <c r="B2" s="5"/>
-      <c r="C2" s="15"/>
-      <c r="D2" s="15"/>
-      <c r="E2" s="15"/>
-      <c r="F2" s="15"/>
-      <c r="G2" s="15"/>
-      <c r="H2" s="15"/>
-      <c r="I2" s="15"/>
-      <c r="J2" s="15"/>
-      <c r="K2" s="15"/>
-      <c r="L2" s="15"/>
-      <c r="M2" s="15"/>
-      <c r="N2" s="15"/>
-      <c r="O2" s="15"/>
-      <c r="P2" s="15"/>
-      <c r="Q2" s="15"/>
-      <c r="R2" s="15"/>
+      <c r="C2" s="9"/>
+      <c r="D2" s="9"/>
+      <c r="E2" s="9"/>
+      <c r="F2" s="9"/>
+      <c r="G2" s="9"/>
+      <c r="H2" s="9"/>
+      <c r="I2" s="9"/>
+      <c r="J2" s="9"/>
+      <c r="K2" s="9"/>
+      <c r="L2" s="9"/>
+      <c r="M2" s="9"/>
+      <c r="N2" s="9"/>
+      <c r="O2" s="9"/>
+      <c r="P2" s="9"/>
+      <c r="Q2" s="9"/>
+      <c r="R2" s="9"/>
     </row>
     <row r="3" spans="1:34" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="35"/>
-      <c r="B3" s="36"/>
-      <c r="C3" s="15"/>
-      <c r="D3" s="15"/>
-      <c r="E3" s="15"/>
-      <c r="F3" s="15"/>
-      <c r="G3" s="15"/>
-      <c r="H3" s="15"/>
-      <c r="I3" s="15"/>
-      <c r="J3" s="15"/>
-      <c r="K3" s="15"/>
-      <c r="L3" s="15"/>
-      <c r="M3" s="15"/>
-      <c r="N3" s="15"/>
-      <c r="O3" s="15"/>
-      <c r="P3" s="15"/>
-      <c r="Q3" s="15"/>
-      <c r="R3" s="15"/>
+      <c r="A3" s="29"/>
+      <c r="B3" s="30"/>
+      <c r="C3" s="9"/>
+      <c r="D3" s="9"/>
+      <c r="E3" s="9"/>
+      <c r="F3" s="9"/>
+      <c r="G3" s="9"/>
+      <c r="H3" s="9"/>
+      <c r="I3" s="9"/>
+      <c r="J3" s="9"/>
+      <c r="K3" s="9"/>
+      <c r="L3" s="9"/>
+      <c r="M3" s="9"/>
+      <c r="N3" s="9"/>
+      <c r="O3" s="9"/>
+      <c r="P3" s="9"/>
+      <c r="Q3" s="9"/>
+      <c r="R3" s="9"/>
     </row>
     <row r="4" spans="1:34" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B4" s="27"/>
-      <c r="C4" s="27"/>
-      <c r="D4" s="27"/>
-      <c r="E4" s="27"/>
-      <c r="F4" s="27"/>
-      <c r="G4" s="27"/>
-      <c r="H4" s="27"/>
-      <c r="I4" s="27"/>
-      <c r="J4" s="27"/>
-      <c r="K4" s="27"/>
-      <c r="L4" s="27"/>
-      <c r="M4" s="27"/>
-      <c r="N4" s="27"/>
-      <c r="O4" s="27"/>
-      <c r="P4" s="27"/>
-      <c r="Q4" s="27"/>
-      <c r="R4" s="27"/>
+      <c r="B4" s="21"/>
+      <c r="C4" s="21"/>
+      <c r="D4" s="21"/>
+      <c r="E4" s="21"/>
+      <c r="F4" s="21"/>
+      <c r="G4" s="21"/>
+      <c r="H4" s="21"/>
+      <c r="I4" s="21"/>
+      <c r="J4" s="21"/>
+      <c r="K4" s="21"/>
+      <c r="L4" s="21"/>
+      <c r="M4" s="21"/>
+      <c r="N4" s="21"/>
+      <c r="O4" s="21"/>
+      <c r="P4" s="21"/>
+      <c r="Q4" s="21"/>
+      <c r="R4" s="21"/>
     </row>
     <row r="5" spans="1:34" s="4" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="20"/>
-      <c r="B5" s="20"/>
-      <c r="C5" s="19"/>
-      <c r="D5" s="19"/>
-      <c r="E5" s="19"/>
-      <c r="F5" s="19"/>
-      <c r="G5" s="19"/>
-      <c r="H5" s="19"/>
-      <c r="I5" s="19"/>
-      <c r="J5" s="19"/>
-      <c r="K5" s="19"/>
-      <c r="L5" s="19"/>
-      <c r="M5" s="19"/>
-      <c r="N5" s="19"/>
-      <c r="O5" s="19"/>
-      <c r="P5" s="16"/>
-      <c r="Q5" s="16"/>
-      <c r="R5" s="16"/>
+      <c r="A5" s="14"/>
+      <c r="B5" s="14"/>
+      <c r="C5" s="13"/>
+      <c r="D5" s="13"/>
+      <c r="E5" s="13"/>
+      <c r="F5" s="13"/>
+      <c r="G5" s="13"/>
+      <c r="H5" s="13"/>
+      <c r="I5" s="13"/>
+      <c r="J5" s="13"/>
+      <c r="K5" s="13"/>
+      <c r="L5" s="13"/>
+      <c r="M5" s="13"/>
+      <c r="N5" s="13"/>
+      <c r="O5" s="13"/>
+      <c r="P5" s="10"/>
+      <c r="Q5" s="10"/>
+      <c r="R5" s="10"/>
     </row>
     <row r="6" spans="1:34" ht="18" x14ac:dyDescent="0.25">
-      <c r="A6" s="20"/>
-      <c r="B6" s="20"/>
+      <c r="A6" s="14"/>
+      <c r="B6" s="14"/>
       <c r="C6" s="2"/>
       <c r="D6" s="2"/>
       <c r="E6" s="2"/>
@@ -1276,26 +1209,26 @@
       <c r="L6" s="2"/>
       <c r="M6" s="2"/>
       <c r="N6" s="2"/>
-      <c r="O6" s="23"/>
+      <c r="O6" s="17"/>
       <c r="P6" s="2"/>
     </row>
     <row r="7" spans="1:34" x14ac:dyDescent="0.25">
-      <c r="C7" s="30"/>
-      <c r="D7" s="30"/>
-      <c r="E7" s="30"/>
-      <c r="F7" s="30"/>
-      <c r="G7" s="30"/>
-      <c r="H7" s="30"/>
-      <c r="I7" s="30"/>
-      <c r="J7" s="30"/>
-      <c r="K7" s="30"/>
-      <c r="L7" s="30"/>
-      <c r="M7" s="30"/>
-      <c r="N7" s="30"/>
-      <c r="O7" s="30"/>
-      <c r="P7" s="28"/>
-      <c r="Q7" s="28"/>
-      <c r="R7" s="28"/>
+      <c r="C7" s="24"/>
+      <c r="D7" s="24"/>
+      <c r="E7" s="24"/>
+      <c r="F7" s="24"/>
+      <c r="G7" s="24"/>
+      <c r="H7" s="24"/>
+      <c r="I7" s="24"/>
+      <c r="J7" s="24"/>
+      <c r="K7" s="24"/>
+      <c r="L7" s="24"/>
+      <c r="M7" s="24"/>
+      <c r="N7" s="24"/>
+      <c r="O7" s="24"/>
+      <c r="P7" s="22"/>
+      <c r="Q7" s="22"/>
+      <c r="R7" s="22"/>
       <c r="S7" s="3"/>
       <c r="T7" s="3"/>
       <c r="U7" s="3"/>
@@ -1314,9 +1247,9 @@
       <c r="AH7" s="3"/>
     </row>
     <row r="8" spans="1:34" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A8" s="34"/>
-      <c r="B8" s="34"/>
-      <c r="C8" s="14"/>
+      <c r="A8" s="28"/>
+      <c r="B8" s="28"/>
+      <c r="C8" s="8"/>
       <c r="D8" s="3"/>
       <c r="E8" s="3"/>
       <c r="F8" s="3"/>
@@ -1326,7 +1259,7 @@
       <c r="J8" s="3"/>
       <c r="K8" s="3"/>
       <c r="L8" s="1"/>
-      <c r="M8" s="29"/>
+      <c r="M8" s="23"/>
       <c r="N8" s="7"/>
       <c r="O8" s="7" t="s">
         <v>6</v>
@@ -1334,114 +1267,114 @@
       <c r="R8" s="6"/>
     </row>
     <row r="9" spans="1:34" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="G9" s="28"/>
-      <c r="H9" s="28"/>
-      <c r="I9" s="28"/>
-      <c r="J9" s="28"/>
-      <c r="K9" s="28"/>
-      <c r="N9" s="17"/>
-      <c r="O9" s="17" t="s">
+      <c r="G9" s="22"/>
+      <c r="H9" s="22"/>
+      <c r="I9" s="22"/>
+      <c r="J9" s="22"/>
+      <c r="K9" s="22"/>
+      <c r="N9" s="11"/>
+      <c r="O9" s="11" t="s">
         <v>7</v>
       </c>
       <c r="P9" s="6"/>
     </row>
     <row r="10" spans="1:34" x14ac:dyDescent="0.25">
-      <c r="G10" s="28"/>
-      <c r="H10" s="28"/>
-      <c r="I10" s="28"/>
-      <c r="J10" s="28"/>
-      <c r="K10" s="28"/>
-      <c r="L10" s="24"/>
-      <c r="P10" s="25"/>
+      <c r="G10" s="22"/>
+      <c r="H10" s="22"/>
+      <c r="I10" s="22"/>
+      <c r="J10" s="22"/>
+      <c r="K10" s="22"/>
+      <c r="L10" s="18"/>
+      <c r="P10" s="19"/>
     </row>
     <row r="11" spans="1:34" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="31" t="s">
+      <c r="A11" s="25" t="s">
         <v>13</v>
       </c>
-      <c r="B11" s="33" t="s">
+      <c r="B11" s="27" t="s">
         <v>3</v>
       </c>
-      <c r="C11" s="33" t="s">
+      <c r="C11" s="27" t="s">
         <v>15</v>
       </c>
-      <c r="D11" s="33" t="s">
+      <c r="D11" s="27" t="s">
         <v>5</v>
       </c>
-      <c r="E11" s="33" t="s">
+      <c r="E11" s="27" t="s">
         <v>14</v>
       </c>
-      <c r="F11" s="33" t="s">
+      <c r="F11" s="27" t="s">
         <v>16</v>
       </c>
-      <c r="G11" s="21"/>
-      <c r="H11" s="21"/>
-      <c r="I11" s="21"/>
-      <c r="J11" s="21"/>
-      <c r="K11" s="21"/>
-      <c r="L11" s="33" t="s">
+      <c r="G11" s="15"/>
+      <c r="H11" s="15"/>
+      <c r="I11" s="15"/>
+      <c r="J11" s="15"/>
+      <c r="K11" s="15"/>
+      <c r="L11" s="27" t="s">
         <v>0</v>
       </c>
-      <c r="M11" s="33" t="s">
+      <c r="M11" s="27" t="s">
         <v>2</v>
       </c>
-      <c r="N11" s="33" t="s">
+      <c r="N11" s="27" t="s">
         <v>1</v>
       </c>
-      <c r="O11" s="33" t="s">
+      <c r="O11" s="27" t="s">
         <v>4</v>
       </c>
-      <c r="P11" s="25"/>
+      <c r="P11" s="19"/>
     </row>
     <row r="12" spans="1:34" ht="75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="32"/>
-      <c r="B12" s="18"/>
-      <c r="C12" s="18"/>
-      <c r="D12" s="18"/>
-      <c r="E12" s="18"/>
-      <c r="F12" s="18"/>
-      <c r="G12" s="18" t="s">
+      <c r="A12" s="26"/>
+      <c r="B12" s="12"/>
+      <c r="C12" s="12"/>
+      <c r="D12" s="12"/>
+      <c r="E12" s="12"/>
+      <c r="F12" s="12"/>
+      <c r="G12" s="12" t="s">
         <v>8</v>
       </c>
-      <c r="H12" s="18" t="s">
+      <c r="H12" s="12" t="s">
         <v>9</v>
       </c>
-      <c r="I12" s="18" t="s">
+      <c r="I12" s="12" t="s">
         <v>10</v>
       </c>
-      <c r="J12" s="18" t="s">
+      <c r="J12" s="12" t="s">
         <v>11</v>
       </c>
-      <c r="K12" s="18" t="s">
+      <c r="K12" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="L12" s="18"/>
-      <c r="M12" s="18"/>
-      <c r="N12" s="18"/>
-      <c r="O12" s="18"/>
+      <c r="L12" s="12"/>
+      <c r="M12" s="12"/>
+      <c r="N12" s="12"/>
+      <c r="O12" s="12"/>
     </row>
     <row r="15" spans="1:34" x14ac:dyDescent="0.25">
-      <c r="L15" s="8"/>
-      <c r="M15" s="9"/>
+      <c r="L15" s="31"/>
+      <c r="M15" s="31"/>
     </row>
     <row r="16" spans="1:34" x14ac:dyDescent="0.25">
-      <c r="L16" s="10"/>
-      <c r="M16" s="11"/>
+      <c r="L16" s="31"/>
+      <c r="M16" s="31"/>
     </row>
     <row r="17" spans="12:13" x14ac:dyDescent="0.25">
-      <c r="L17" s="8"/>
-      <c r="M17" s="9"/>
+      <c r="L17" s="31"/>
+      <c r="M17" s="31"/>
     </row>
     <row r="18" spans="12:13" x14ac:dyDescent="0.25">
-      <c r="L18" s="10"/>
-      <c r="M18" s="11"/>
+      <c r="L18" s="31"/>
+      <c r="M18" s="31"/>
     </row>
     <row r="19" spans="12:13" x14ac:dyDescent="0.25">
-      <c r="L19" s="12"/>
-      <c r="M19" s="13"/>
+      <c r="L19" s="31"/>
+      <c r="M19" s="31"/>
     </row>
     <row r="20" spans="12:13" x14ac:dyDescent="0.25">
-      <c r="L20" s="12"/>
-      <c r="M20" s="13"/>
+      <c r="L20" s="31"/>
+      <c r="M20" s="31"/>
     </row>
   </sheetData>
   <pageMargins left="0.26" right="0.23" top="0.43" bottom="0.33" header="0.17" footer="0.17"/>

</xml_diff>